<commit_message>
Auto sync live scraped sales control data and fresh sold transactions: 2026-08-03 11:42:32
</commit_message>
<xml_diff>
--- a/files/九龙-何文田-Prince Central.xlsx
+++ b/files/九龙-何文田-Prince Central.xlsx
@@ -789,7 +789,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>2022-07-04</t>
+          <t>2022-07-05</t>
         </is>
       </c>
       <c r="H3" s="5" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2022-07-19</t>
+          <t>2022-07-20</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2023-03-23</t>
+          <t>2023-03-24</t>
         </is>
       </c>
       <c r="H6" s="5" t="n">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="H8" s="5" t="n">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>2024-07-10</t>
+          <t>2024-07-11</t>
         </is>
       </c>
       <c r="H9" s="5" t="n">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="H18" s="5" t="n">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="H23" s="5" t="n">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>2022-06-28</t>
+          <t>2022-06-29</t>
         </is>
       </c>
       <c r="H27" s="5" t="n">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>2022-07-12</t>
+          <t>2022-07-13</t>
         </is>
       </c>
       <c r="H29" s="5" t="n">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>2022-06-23</t>
+          <t>2022-06-24</t>
         </is>
       </c>
       <c r="H30" s="5" t="n">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>2023-12-10</t>
+          <t>2023-12-11</t>
         </is>
       </c>
       <c r="H32" s="5" t="n">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>2025-05-19</t>
+          <t>2025-05-20</t>
         </is>
       </c>
       <c r="H34" s="5" t="n">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>2023-06-18</t>
+          <t>2023-06-19</t>
         </is>
       </c>
       <c r="H37" s="5" t="n">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>2022-06-29</t>
+          <t>2022-06-30</t>
         </is>
       </c>
       <c r="H39" s="5" t="n">
@@ -3265,7 +3265,7 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2022-06-17</t>
         </is>
       </c>
       <c r="H41" s="5" t="n">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2022-06-17</t>
         </is>
       </c>
       <c r="H42" s="5" t="n">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>2023-05-17</t>
+          <t>2023-05-18</t>
         </is>
       </c>
       <c r="H45" s="5" t="n">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>2024-09-25</t>
+          <t>2024-09-26</t>
         </is>
       </c>
       <c r="H47" s="5" t="n">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>2022-06-19</t>
+          <t>2022-06-20</t>
         </is>
       </c>
       <c r="H49" s="5" t="n">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2022-06-17</t>
         </is>
       </c>
       <c r="H53" s="5" t="n">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>2022-06-21</t>
+          <t>2022-06-22</t>
         </is>
       </c>
       <c r="H61" s="5" t="n">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>2022-06-23</t>
+          <t>2022-06-24</t>
         </is>
       </c>
       <c r="H63" s="5" t="n">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>2022-11-16</t>
+          <t>2022-11-17</t>
         </is>
       </c>
       <c r="H65" s="5" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2022-06-17</t>
         </is>
       </c>
       <c r="H69" s="5" t="n">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>2022-07-10</t>
+          <t>2022-07-11</t>
         </is>
       </c>
       <c r="H74" s="5" t="n">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>2022-07-27</t>
+          <t>2022-07-28</t>
         </is>
       </c>
       <c r="H77" s="5" t="n">
@@ -5785,7 +5785,7 @@
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>2024-06-17</t>
+          <t>2024-06-18</t>
         </is>
       </c>
       <c r="H81" s="5" t="n">
@@ -6033,7 +6033,7 @@
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>2022-07-04</t>
+          <t>2022-07-05</t>
         </is>
       </c>
       <c r="H85" s="5" t="n">
@@ -6537,7 +6537,7 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>2022-06-23</t>
+          <t>2022-06-24</t>
         </is>
       </c>
       <c r="H93" s="5" t="n">
@@ -7386,7 +7386,7 @@
           <t>B | 1351呎 (4+房)
 $6008万
 $44,474/呎
-(22年-07月-04日)</t>
+(22年-07月-05日)</t>
         </is>
       </c>
       <c r="D5" s="22" t="inlineStr"/>
@@ -7415,7 +7415,7 @@
           <t>B | 685呎 (3房)
 $2460万
 $35,907/呎
-(23年-03月-23日)</t>
+(23年-03月-24日)</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
@@ -7423,7 +7423,7 @@
           <t>C | 890呎 (4+房)
 $3218万
 $36,154/呎
-(22年-07月-19日)</t>
+(22年-07月-20日)</t>
         </is>
       </c>
       <c r="E6" s="22" t="inlineStr"/>
@@ -7459,7 +7459,7 @@
           <t>C | 344呎 (1房)
 $1075万
 $31,255/呎
-(24年-07月-10日)</t>
+(24年-07月-11日)</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
@@ -7467,7 +7467,7 @@
           <t>D | 891呎 (4+房)
 $3150万
 $35,354/呎
-(26年-03月-03日)</t>
+(26年-03月-04日)</t>
         </is>
       </c>
       <c r="F7" s="22" t="inlineStr"/>
@@ -7486,7 +7486,7 @@
           <t>A | 436呎 (2房)
 $1388万
 $31,838/呎
-(26年-04月-27日)</t>
+(26年-04月-28日)</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
@@ -7566,7 +7566,7 @@
           <t>C | 304呎 (1房)
 $971万
 $31,950/呎
-(26年-06月-17日)</t>
+(26年-06月-18日)</t>
         </is>
       </c>
       <c r="E9" s="25" t="inlineStr">
@@ -7614,7 +7614,7 @@
           <t>A | 436呎 (2房)
 $1312万
 $30,095/呎
-(23年-12月-10日)</t>
+(23年-12月-11日)</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
@@ -7630,7 +7630,7 @@
           <t>C | 303呎 (1房)
 $962万
 $31,739/呎
-(22年-06月-23日)</t>
+(22年-06月-24日)</t>
         </is>
       </c>
       <c r="E10" s="21" t="inlineStr">
@@ -7638,7 +7638,7 @@
           <t>D | 345呎 (1房)
 $1060万
 $30,738/呎
-(22年-07月-12日)</t>
+(22年-07月-13日)</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
@@ -7654,7 +7654,7 @@
           <t>F | 624呎 (3房)
 $2132万
 $34,173/呎
-(22年-06月-28日)</t>
+(22年-06月-29日)</t>
         </is>
       </c>
       <c r="H10" s="23" t="inlineStr">
@@ -7678,7 +7678,7 @@
           <t>A | 436呎 (2房)
 $1302万
 $29,855/呎
-(22年-06月-29日)</t>
+(22年-06月-30日)</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
@@ -7694,7 +7694,7 @@
           <t>C | 304呎 (1房)
 $946万
 $31,106/呎
-(23年-06月-18日)</t>
+(23年-06月-19日)</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
@@ -7718,7 +7718,7 @@
           <t>F | 624呎 (3房)
 $2062万
 $33,049/呎
-(25年-05月-19日)</t>
+(25年-05月-20日)</t>
         </is>
       </c>
       <c r="H11" s="24" t="inlineStr">
@@ -7742,7 +7742,7 @@
           <t>A | 436呎 (2房)
 $1362万
 $31,238/呎
-(24年-09月-25日)</t>
+(24年-09月-26日)</t>
         </is>
       </c>
       <c r="C12" s="23" t="inlineStr">
@@ -7758,7 +7758,7 @@
           <t>C | 304呎 (1房)
 $924万
 $30,401/呎
-(23年-05月-17日)</t>
+(23年-05月-18日)</t>
         </is>
       </c>
       <c r="E12" s="25" t="inlineStr">
@@ -7782,7 +7782,7 @@
           <t>F | 338呎 (1房)
 $1032万
 $30,527/呎
-(22年-06月-16日)</t>
+(22年-06月-17日)</t>
         </is>
       </c>
       <c r="H12" s="21" t="inlineStr">
@@ -7790,7 +7790,7 @@
           <t>G | 344呎 (1房)
 $1042万
 $30,301/呎
-(22年-06月-16日)</t>
+(22年-06月-17日)</t>
         </is>
       </c>
       <c r="I12" s="25" t="inlineStr">
@@ -7829,7 +7829,7 @@
           <t>C | 303呎 (1房)
 $896万
 $29,573/呎
-(22年-06月-16日)</t>
+(22年-06月-17日)</t>
         </is>
       </c>
       <c r="E13" s="25" t="inlineStr">
@@ -7861,7 +7861,7 @@
           <t>G | 344呎 (1房)
 $1034万
 $30,059/呎
-(22年-06月-19日)</t>
+(22年-06月-20日)</t>
         </is>
       </c>
       <c r="I13" s="25" t="inlineStr">
@@ -7884,7 +7884,7 @@
           <t>A | 436呎 (2房)
 $1273万
 $29,208/呎
-(22年-06月-23日)</t>
+(22年-06月-24日)</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
@@ -7900,7 +7900,7 @@
           <t>C | 303呎 (1房)
 $893万
 $29,461/呎
-(22年-06月-21日)</t>
+(22年-06月-22日)</t>
         </is>
       </c>
       <c r="E14" s="25" t="inlineStr">
@@ -7971,7 +7971,7 @@
           <t>C | 303呎 (1房)
 $893万
 $29,461/呎
-(22年-06月-16日)</t>
+(22年-06月-17日)</t>
         </is>
       </c>
       <c r="E15" s="24" t="inlineStr">
@@ -8003,7 +8003,7 @@
           <t>G | 343呎 (1房)
 $1031万
 $30,060/呎
-(22年-11月-16日)</t>
+(22年-11月-17日)</t>
         </is>
       </c>
       <c r="I15" s="25" t="inlineStr">
@@ -8042,7 +8042,7 @@
           <t>C | 303呎 (1房)
 $886万
 $29,239/呎
-(22年-07月-27日)</t>
+(22年-07月-28日)</t>
         </is>
       </c>
       <c r="E16" s="25" t="inlineStr">
@@ -8066,7 +8066,7 @@
           <t>F | 338呎 (1房)
 $1015万
 $30,017/呎
-(22年-07月-10日)</t>
+(22年-07月-11日)</t>
         </is>
       </c>
       <c r="H16" s="25" t="inlineStr">
@@ -8113,7 +8113,7 @@
           <t>C | 303呎 (1房)
 $883万
 $29,141/呎
-(22年-07月-04日)</t>
+(22年-07月-05日)</t>
         </is>
       </c>
       <c r="E17" s="25" t="inlineStr">
@@ -8145,7 +8145,7 @@
           <t>G | 343呎 (1房)
 $1022万
 $29,787/呎
-(24年-06月-17日)</t>
+(24年-06月-18日)</t>
         </is>
       </c>
       <c r="I17" s="24" t="inlineStr">
@@ -8184,7 +8184,7 @@
           <t>C | 303呎 (1房)
 $880万
 $29,043/呎
-(22年-06月-23日)</t>
+(22年-06月-24日)</t>
         </is>
       </c>
       <c r="E18" s="25" t="inlineStr">

</xml_diff>